<commit_message>
finished untill the upload
</commit_message>
<xml_diff>
--- a/data/Final Template.xlsx
+++ b/data/Final Template.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="360" windowWidth="11736" windowHeight="12708" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -25,7 +25,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -40,12 +40,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -56,11 +52,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0000FF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,10 +67,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -87,9 +77,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,38 +476,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="4.21875" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
-    <col width="18.44140625" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
-    <col width="20" bestFit="1" customWidth="1" style="4" min="3" max="3"/>
-    <col width="9.77734375" bestFit="1" customWidth="1" style="4" min="4" max="4"/>
-    <col width="9.44140625" bestFit="1" customWidth="1" style="4" min="5" max="5"/>
-    <col width="9.88671875" bestFit="1" customWidth="1" style="4" min="6" max="6"/>
-    <col width="13.5546875" bestFit="1" customWidth="1" style="4" min="7" max="7"/>
-    <col width="15.77734375" customWidth="1" style="4" min="8" max="8"/>
+    <col width="18.44140625" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
+    <col width="20" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
+    <col width="9.77734375" bestFit="1" customWidth="1" style="3" min="4" max="4"/>
+    <col width="9.44140625" bestFit="1" customWidth="1" style="3" min="5" max="5"/>
+    <col width="9.88671875" bestFit="1" customWidth="1" style="3" min="6" max="6"/>
+    <col width="13.5546875" bestFit="1" customWidth="1" style="3" min="7" max="7"/>
+    <col width="21.21875" customWidth="1" style="3" min="8" max="8"/>
+    <col width="17.21875" customWidth="1" style="3" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Mobileuma ction item overview - 03/10/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>P2P</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>From Angnelo Sheet</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Internal Action item</t>
         </is>
@@ -566,56 +550,88 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
-    <row r="5"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P2P</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RTR</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="6">
-      <c r="D6" s="6" t="n">
-        <v>58</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>R2R</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="H7" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="D7" s="1" t="n"/>
+      <c r="E7" s="1" t="n"/>
+      <c r="F7" s="1" t="n"/>
+      <c r="G7" s="1" t="n"/>
+      <c r="H7" s="1" t="n"/>
+      <c r="I7" s="1" t="n"/>
+      <c r="J7" s="1" t="n"/>
+    </row>
+    <row r="8">
+      <c r="D8" s="1" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="n"/>
+      <c r="H8" s="1" t="n"/>
+      <c r="I8" s="1" t="n"/>
+      <c r="J8" s="1" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="D2:H2"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="A2:A6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add the extra sheet
</commit_message>
<xml_diff>
--- a/data/Final Template.xlsx
+++ b/data/Final Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="360" windowWidth="11736" windowHeight="12708" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="360" windowWidth="23256" windowHeight="6408" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -25,7 +25,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -40,8 +40,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -52,6 +61,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0000FF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,9 +81,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -77,8 +93,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,33 +493,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="18.44140625" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
-    <col width="20" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
-    <col width="9.77734375" bestFit="1" customWidth="1" style="3" min="4" max="4"/>
-    <col width="9.44140625" bestFit="1" customWidth="1" style="3" min="5" max="5"/>
-    <col width="9.88671875" bestFit="1" customWidth="1" style="3" min="6" max="6"/>
-    <col width="13.5546875" bestFit="1" customWidth="1" style="3" min="7" max="7"/>
-    <col width="21.21875" customWidth="1" style="3" min="8" max="8"/>
-    <col width="17.21875" customWidth="1" style="3" min="9" max="9"/>
+    <col width="34.77734375" customWidth="1" style="5" min="1" max="1"/>
+    <col width="18.44140625" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
+    <col width="20" bestFit="1" customWidth="1" style="5" min="3" max="3"/>
+    <col width="9.77734375" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
+    <col width="9.44140625" bestFit="1" customWidth="1" style="5" min="5" max="5"/>
+    <col width="9.88671875" bestFit="1" customWidth="1" style="5" min="6" max="6"/>
+    <col width="13.5546875" bestFit="1" customWidth="1" style="5" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Mobileuma ction item overview - 03/10/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>From Angnelo Sheet</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Internal Action item</t>
         </is>
@@ -539,16 +555,6 @@
           <t>Pending Review</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sent to Mobileum Review  </t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Testing</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -556,22 +562,22 @@
           <t>P2P</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="7" t="n">
         <v>58</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -581,55 +587,172 @@
           <t>RTR</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="D6" s="1" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="1" t="n"/>
-      <c r="H6" s="1" t="n"/>
-      <c r="I6" s="1" t="n"/>
-      <c r="J6" s="1" t="n"/>
-    </row>
-    <row r="7">
-      <c r="D7" s="1" t="n"/>
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="1" t="n"/>
-      <c r="G7" s="1" t="n"/>
-      <c r="H7" s="1" t="n"/>
-      <c r="I7" s="1" t="n"/>
-      <c r="J7" s="1" t="n"/>
-    </row>
-    <row r="8">
-      <c r="D8" s="1" t="n"/>
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="n"/>
-      <c r="G8" s="1" t="n"/>
-      <c r="H8" s="1" t="n"/>
-      <c r="I8" s="1" t="n"/>
-      <c r="J8" s="1" t="n"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Count of Sr. No</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Column Labels</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Row Labels</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CRP</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CRP2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FRD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Go live</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Pending - Mobileum</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pending - Zenardy</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>42</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B1:J1"/>
     <mergeCell ref="D2:H2"/>
     <mergeCell ref="B2:C2"/>
   </mergeCells>

</xml_diff>